<commit_message>
feat: clean DAINESE templates + rewrite debit generator with formula support
- Clean 5 DAINESE templates (remove old data, keep reference row with formulas)
- Split generator into 3 modules: orchestrator, data-resolver, template-filler
- Formula injection with row adjustment (V=SUM(K{row}:U{row}), etc.)
- Totals row auto-adjusts SUM range
- Filter jobs by scheduled_date instead of created_at
</commit_message>
<xml_diff>
--- a/stored_files/templates/DAINESE/DAINESE_CO_template.xlsx
+++ b/stored_files/templates/DAINESE/DAINESE_CO_template.xlsx
@@ -1277,7 +1277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.08984375" defaultRowHeight="14"/>
   <cols>
     <col width="5.36328125" customWidth="1" style="69" min="1" max="1"/>
@@ -1326,7 +1326,6 @@
     <row r="4">
       <c r="A4" s="69" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="68" t="inlineStr">
         <is>
@@ -1337,7 +1336,6 @@
     <row r="7">
       <c r="A7" s="69" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
@@ -1506,46 +1504,53 @@
       </c>
     </row>
     <row r="16" ht="18.5" customFormat="1" customHeight="1" s="33" thickBot="1">
-      <c r="A16" s="53" t="n"/>
-      <c r="B16" s="60" t="n"/>
-      <c r="C16" s="61" t="n"/>
-      <c r="D16" s="61" t="n"/>
-      <c r="E16" s="54" t="n"/>
-      <c r="F16" s="55" t="n"/>
-      <c r="G16" s="56" t="n"/>
-      <c r="H16" s="56" t="n"/>
-      <c r="I16" s="84" t="n"/>
-      <c r="J16" s="54" t="n"/>
-      <c r="K16" s="55" t="n"/>
-      <c r="L16" s="56" t="n"/>
-      <c r="M16" s="57" t="n"/>
+      <c r="A16" s="76" t="inlineStr">
+        <is>
+          <t>TỔNG TRƯỚC VAT</t>
+        </is>
+      </c>
+      <c r="B16" s="85" t="n"/>
+      <c r="C16" s="85" t="n"/>
+      <c r="D16" s="85" t="n"/>
+      <c r="E16" s="85" t="n"/>
+      <c r="F16" s="85" t="n"/>
+      <c r="G16" s="86" t="n"/>
+      <c r="H16" s="45">
+        <f>SUM(H15:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="46" t="n"/>
+      <c r="J16" s="47" t="n"/>
+      <c r="K16" s="47" t="n"/>
+      <c r="L16" s="47">
+        <f>SUM(L15:L15)</f>
+        <v/>
+      </c>
+      <c r="M16" s="48" t="n"/>
     </row>
     <row r="17" ht="19" customFormat="1" customHeight="1" s="33">
-      <c r="A17" s="76" t="inlineStr">
-        <is>
-          <t>TỔNG TRƯỚC VAT</t>
-        </is>
-      </c>
-      <c r="B17" s="85" t="n"/>
-      <c r="C17" s="85" t="n"/>
-      <c r="D17" s="85" t="n"/>
-      <c r="E17" s="85" t="n"/>
-      <c r="F17" s="85" t="n"/>
-      <c r="G17" s="86" t="n"/>
-      <c r="H17" s="45">
-        <f>SUM(H15:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="46" t="n"/>
-      <c r="J17" s="47" t="n"/>
-      <c r="K17" s="47" t="n"/>
-      <c r="L17" s="47" t="n"/>
-      <c r="M17" s="48" t="n"/>
+      <c r="A17" s="78" t="inlineStr">
+        <is>
+          <t>VAT (0%)</t>
+        </is>
+      </c>
+      <c r="B17" s="87" t="n"/>
+      <c r="C17" s="87" t="n"/>
+      <c r="D17" s="87" t="n"/>
+      <c r="E17" s="87" t="n"/>
+      <c r="F17" s="87" t="n"/>
+      <c r="G17" s="88" t="n"/>
+      <c r="H17" s="34" t="n"/>
+      <c r="I17" s="35" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="9" t="n"/>
+      <c r="M17" s="31" t="n"/>
     </row>
     <row r="18" ht="19" customFormat="1" customHeight="1" s="33">
       <c r="A18" s="78" t="inlineStr">
         <is>
-          <t>VAT (0%)</t>
+          <t>TỔNG SAU VAT</t>
         </is>
       </c>
       <c r="B18" s="87" t="n"/>
@@ -1554,67 +1559,60 @@
       <c r="E18" s="87" t="n"/>
       <c r="F18" s="87" t="n"/>
       <c r="G18" s="88" t="n"/>
-      <c r="H18" s="34" t="n"/>
+      <c r="H18" s="34">
+        <f>H16+H17</f>
+        <v/>
+      </c>
       <c r="I18" s="35" t="n"/>
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="9" t="n"/>
-      <c r="L18" s="9" t="n"/>
+      <c r="L18" s="36">
+        <f>SUM(L15:L15)</f>
+        <v/>
+      </c>
       <c r="M18" s="31" t="n"/>
     </row>
     <row r="19" ht="19" customFormat="1" customHeight="1" s="33">
-      <c r="A19" s="78" t="inlineStr">
-        <is>
-          <t>TỔNG SAU VAT</t>
-        </is>
-      </c>
-      <c r="B19" s="87" t="n"/>
-      <c r="C19" s="87" t="n"/>
-      <c r="D19" s="87" t="n"/>
-      <c r="E19" s="87" t="n"/>
-      <c r="F19" s="87" t="n"/>
-      <c r="G19" s="88" t="n"/>
-      <c r="H19" s="34">
-        <f>H17+H18</f>
+      <c r="A19" s="70" t="inlineStr">
+        <is>
+          <t>TỔNG THANH TOÁN</t>
+        </is>
+      </c>
+      <c r="B19" s="89" t="n"/>
+      <c r="C19" s="89" t="n"/>
+      <c r="D19" s="89" t="n"/>
+      <c r="E19" s="89" t="n"/>
+      <c r="F19" s="89" t="n"/>
+      <c r="G19" s="89" t="n"/>
+      <c r="H19" s="90" t="n"/>
+      <c r="I19" s="91">
+        <f>H18+L18</f>
         <v/>
       </c>
-      <c r="I19" s="35" t="n"/>
-      <c r="J19" s="9" t="n"/>
-      <c r="K19" s="9" t="n"/>
-      <c r="L19" s="36">
-        <f>SUM(L15:L16)</f>
-        <v/>
-      </c>
-      <c r="M19" s="31" t="n"/>
+      <c r="J19" s="89" t="n"/>
+      <c r="K19" s="89" t="n"/>
+      <c r="L19" s="89" t="n"/>
+      <c r="M19" s="92" t="n"/>
+      <c r="N19" s="37" t="n"/>
     </row>
     <row r="20" ht="19" customFormat="1" customHeight="1" s="33" thickBot="1">
-      <c r="A20" s="70" t="inlineStr">
-        <is>
-          <t>TỔNG THANH TOÁN</t>
-        </is>
-      </c>
-      <c r="B20" s="89" t="n"/>
-      <c r="C20" s="89" t="n"/>
-      <c r="D20" s="89" t="n"/>
-      <c r="E20" s="89" t="n"/>
-      <c r="F20" s="89" t="n"/>
-      <c r="G20" s="89" t="n"/>
-      <c r="H20" s="90" t="n"/>
-      <c r="I20" s="91">
-        <f>H19+L19</f>
-        <v/>
-      </c>
-      <c r="J20" s="89" t="n"/>
-      <c r="K20" s="89" t="n"/>
-      <c r="L20" s="89" t="n"/>
-      <c r="M20" s="92" t="n"/>
-      <c r="N20" s="37" t="n"/>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Tổng số tiền bằng chữ: Một triệu hai trăm sáu mươi nghìn đồng chẵn.,/</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="20" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="5" t="n"/>
     </row>
     <row r="21" ht="21" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Tổng số tiền bằng chữ: Một triệu hai trăm sáu mươi nghìn đồng chẵn.,/</t>
-        </is>
-      </c>
+      <c r="A21" s="21" t="n"/>
       <c r="B21" s="14" t="n"/>
       <c r="C21" s="15" t="n"/>
       <c r="D21" s="16" t="n"/>
@@ -1623,44 +1621,37 @@
       <c r="G21" s="19" t="n"/>
       <c r="H21" s="20" t="n"/>
       <c r="I21" s="16" t="n"/>
-      <c r="J21" s="5" t="n"/>
     </row>
     <row r="22" ht="21" customHeight="1">
-      <c r="A22" s="21" t="n"/>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="20" t="n"/>
-      <c r="I22" s="16" t="n"/>
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH DAINESE VIỆT NAM</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="25" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="H22" s="27" t="inlineStr">
+        <is>
+          <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ 5P VIỆT NAM</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="21" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
-        <is>
-          <t>CÔNG TY TNHH DAINESE VIỆT NAM</t>
-        </is>
-      </c>
-      <c r="B23" s="23" t="n"/>
-      <c r="C23" s="22" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="25" t="n"/>
-      <c r="F23" s="26" t="n"/>
-      <c r="H23" s="27" t="inlineStr">
-        <is>
-          <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ 5P VIỆT NAM</t>
-        </is>
-      </c>
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="75" t="n"/>
     </row>
     <row r="24" ht="21" customHeight="1">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="75" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="G25" s="2" t="n"/>
@@ -1693,27 +1684,35 @@
       <c r="I30" s="2" t="n"/>
     </row>
     <row r="31" ht="1.5" customHeight="1">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>Thông tin chuyển khoản:</t>
+        </is>
+      </c>
+      <c r="B31" s="39" t="n"/>
+      <c r="C31" s="40" t="n"/>
+      <c r="D31" s="24" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
     </row>
     <row r="32" ht="15.5" customHeight="1">
-      <c r="A32" s="38" t="inlineStr">
-        <is>
-          <t>Thông tin chuyển khoản:</t>
+      <c r="A32" s="40" t="inlineStr">
+        <is>
+          <t>Tài khoản: Công Ty TNHH Thương mại và dịch vụ 5P Việt Nam</t>
         </is>
       </c>
       <c r="B32" s="39" t="n"/>
       <c r="C32" s="40" t="n"/>
       <c r="D32" s="24" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
+      <c r="G32" s="3" t="n"/>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n"/>
     </row>
     <row r="33" ht="15.5" customHeight="1">
       <c r="A33" s="40" t="inlineStr">
         <is>
-          <t>Tài khoản: Công Ty TNHH Thương mại và dịch vụ 5P Việt Nam</t>
+          <t>Số tài khoản: 346886</t>
         </is>
       </c>
       <c r="B33" s="39" t="n"/>
@@ -1724,29 +1723,17 @@
       <c r="I33" s="3" t="n"/>
     </row>
     <row r="34" ht="15.5" customHeight="1">
-      <c r="A34" s="40" t="inlineStr">
-        <is>
-          <t>Số tài khoản: 346886</t>
-        </is>
-      </c>
-      <c r="B34" s="39" t="n"/>
-      <c r="C34" s="40" t="n"/>
-      <c r="D34" s="24" t="n"/>
+      <c r="A34" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tại Ngân hàng: Ngân hàng TMCP Kỹ thương Việt Nam - Techcombank Chi nhánh Đông Đô
+ </t>
+        </is>
+      </c>
       <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
     </row>
-    <row r="35" ht="15.5" customHeight="1">
-      <c r="A35" s="74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tại Ngân hàng: Ngân hàng TMCP Kỹ thương Việt Nam - Techcombank Chi nhánh Đông Đô
- </t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-    </row>
+    <row r="35" ht="15.5" customHeight="1"/>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="H24:J24"/>

</xml_diff>